<commit_message>
Film 2: Brain in a Vat
- Descartes' evil demon (1641) → Putnam's brain in a vat (1981): the skeptic's argument, Putnam's
  semantic-externalist reply, the recent-envatment objection and Nagel's worry
- Floating 'experienced world' above the lab, glitch reveal hook, Descartes' firelit study with the demon
- Engine: table/bench/house kit, glitch overlay, thought-bubble labels, numbered-steps card
- Catalogue: Brain in a Vat marked created with its video essay; fixed broken SEP links
  (Brain in a Vat → Content Externalism and Skepticism; Floating Man → Arabic and Islamic Philosophy of Mind)
- Guide: label offsets in scaled groups, name pronunciation checks, verify SEP links
</commit_message>
<xml_diff>
--- a/thought_experiments.xlsx
+++ b/thought_experiments.xlsx
@@ -594,7 +594,7 @@
           <t>Brain in a Vat</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -617,7 +617,7 @@
         <f>AVERAGE(D2:F2)</f>
         <v/>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -632,9 +632,13 @@
           <t>Putnam, Reason, Truth and History (1981)</t>
         </is>
       </c>
-      <c r="K2" s="13" t="n"/>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Video essay</t>
+        </is>
+      </c>
       <c r="L2" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -643,7 +647,7 @@
           <t>Fermi Paradox</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -666,7 +670,7 @@
         <f>AVERAGE(D3:F3)</f>
         <v/>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -692,7 +696,7 @@
           <t>Grandfather Paradox</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -711,7 +715,7 @@
         <f>AVERAGE(D4:F4)</f>
         <v/>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -737,7 +741,7 @@
           <t>Infinite Monkey Theorem</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -756,7 +760,7 @@
         <f>AVERAGE(D5:F5)</f>
         <v/>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -782,7 +786,7 @@
           <t>Plato's Cave</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -801,7 +805,7 @@
         <f>AVERAGE(D6:F6)</f>
         <v/>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -827,7 +831,7 @@
           <t>Ship of Theseus</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -850,7 +854,7 @@
         <f>AVERAGE(D7:F7)</f>
         <v/>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -876,7 +880,7 @@
           <t>Simulation Argument</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -899,7 +903,7 @@
         <f>AVERAGE(D8:F8)</f>
         <v/>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -925,7 +929,7 @@
           <t>Tragedy of the Commons</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
@@ -944,7 +948,7 @@
         <f>AVERAGE(D9:F9)</f>
         <v/>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -970,7 +974,7 @@
           <t>Tree Falling in a Forest</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -989,7 +993,7 @@
         <f>AVERAGE(D10:F10)</f>
         <v/>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1015,7 +1019,7 @@
           <t>Trolley Problem</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -1038,7 +1042,7 @@
         <f>AVERAGE(D11:F11)</f>
         <v/>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1068,7 +1072,7 @@
           <t>Chinese Room</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -1087,7 +1091,7 @@
         <f>AVERAGE(D12:F12)</f>
         <v/>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1113,7 +1117,7 @@
           <t>Monty Hall Problem</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -1132,7 +1136,7 @@
         <f>AVERAGE(D13:F13)</f>
         <v/>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1158,7 +1162,7 @@
           <t>Schrödinger's Cat</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -1177,7 +1181,7 @@
         <f>AVERAGE(D14:F14)</f>
         <v/>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1203,7 +1207,7 @@
           <t>Prisoner's Dilemma</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -1222,7 +1226,7 @@
         <f>AVERAGE(D15:F15)</f>
         <v/>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1248,7 +1252,7 @@
           <t>Turing Test</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
@@ -1267,7 +1271,7 @@
         <f>AVERAGE(D16:F16)</f>
         <v/>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1293,7 +1297,7 @@
           <t>Achilles and the Tortoise</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -1312,7 +1316,7 @@
         <f>AVERAGE(D17:F17)</f>
         <v/>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1338,7 +1342,7 @@
           <t>Blind Men and an Elephant</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -1357,7 +1361,7 @@
         <f>AVERAGE(D18:F18)</f>
         <v/>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1383,7 +1387,7 @@
           <t>Dark Forest</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -1406,7 +1410,7 @@
         <f>AVERAGE(D19:F19)</f>
         <v/>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1432,7 +1436,7 @@
           <t>Drowning Child</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -1451,7 +1455,7 @@
         <f>AVERAGE(D20:F20)</f>
         <v/>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1477,7 +1481,7 @@
           <t>Experience Machine</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -1496,7 +1500,7 @@
         <f>AVERAGE(D21:F21)</f>
         <v/>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1522,7 +1526,7 @@
           <t>Footbridge (Fat Man)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -1545,7 +1549,7 @@
         <f>AVERAGE(D22:F22)</f>
         <v/>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1571,7 +1575,7 @@
           <t>Heraclitus's River</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -1594,7 +1598,7 @@
         <f>AVERAGE(D23:F23)</f>
         <v/>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1620,7 +1624,7 @@
           <t>Mary's Room</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -1639,7 +1643,7 @@
         <f>AVERAGE(D24:F24)</f>
         <v/>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H24" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1665,7 +1669,7 @@
           <t>Omelas</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -1684,7 +1688,7 @@
         <f>AVERAGE(D25:F25)</f>
         <v/>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1710,7 +1714,7 @@
           <t>Paperclip Maximizer</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
@@ -1729,7 +1733,7 @@
         <f>AVERAGE(D26:F26)</f>
         <v/>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1755,7 +1759,7 @@
           <t>Ring of Gyges</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -1774,7 +1778,7 @@
         <f>AVERAGE(D27:F27)</f>
         <v/>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H27" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1800,7 +1804,7 @@
           <t>Russell's Teapot</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -1819,7 +1823,7 @@
         <f>AVERAGE(D28:F28)</f>
         <v/>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1845,7 +1849,7 @@
           <t>Turtles All the Way Down</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -1868,7 +1872,7 @@
         <f>AVERAGE(D29:F29)</f>
         <v/>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H29" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1894,7 +1898,7 @@
           <t>Watchmaker Analogy</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -1913,7 +1917,7 @@
         <f>AVERAGE(D30:F30)</f>
         <v/>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H30" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1939,7 +1943,7 @@
           <t>Great Filter</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -1962,7 +1966,7 @@
         <f>AVERAGE(D31:F31)</f>
         <v/>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="H31" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -1988,7 +1992,7 @@
           <t>Hilbert's Hotel</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -2007,7 +2011,7 @@
         <f>AVERAGE(D32:F32)</f>
         <v/>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="H32" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2033,7 +2037,7 @@
           <t>Maxwell's Demon</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -2052,7 +2056,7 @@
         <f>AVERAGE(D33:F33)</f>
         <v/>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H33" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2078,7 +2082,7 @@
           <t>Twin Paradox</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -2097,7 +2101,7 @@
         <f>AVERAGE(D34:F34)</f>
         <v/>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H34" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2123,7 +2127,7 @@
           <t>Evil Demon</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -2146,7 +2150,7 @@
         <f>AVERAGE(D35:F35)</f>
         <v/>
       </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="H35" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2172,7 +2176,7 @@
           <t>Omnipotence Paradox (the Stone)</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -2191,7 +2195,7 @@
         <f>AVERAGE(D36:F36)</f>
         <v/>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H36" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2217,7 +2221,7 @@
           <t>State of Nature</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Political Philosophy</t>
         </is>
@@ -2236,7 +2240,7 @@
         <f>AVERAGE(D37:F37)</f>
         <v/>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H37" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2262,7 +2266,7 @@
           <t>Broken Window</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
@@ -2281,7 +2285,7 @@
         <f>AVERAGE(D38:F38)</f>
         <v/>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H38" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2307,7 +2311,7 @@
           <t>Buridan's Ass</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -2326,7 +2330,7 @@
         <f>AVERAGE(D39:F39)</f>
         <v/>
       </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="H39" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2352,7 +2356,7 @@
           <t>Butterfly Dream</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -2375,7 +2379,7 @@
         <f>AVERAGE(D40:F40)</f>
         <v/>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H40" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2401,7 +2405,7 @@
           <t>Chesterton's Fence</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>Political Philosophy</t>
         </is>
@@ -2420,7 +2424,7 @@
         <f>AVERAGE(D41:F41)</f>
         <v/>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="H41" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2446,7 +2450,7 @@
           <t>Douglas Adams's Puddle</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -2469,7 +2473,7 @@
         <f>AVERAGE(D42:F42)</f>
         <v/>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H42" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2495,7 +2499,7 @@
           <t>Flatland</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -2514,7 +2518,7 @@
         <f>AVERAGE(D43:F43)</f>
         <v/>
       </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="H43" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2540,7 +2544,7 @@
           <t>Galileo's Falling Bodies</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -2559,7 +2563,7 @@
         <f>AVERAGE(D44:F44)</f>
         <v/>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="H44" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2585,7 +2589,7 @@
           <t>Gray Goo</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
@@ -2604,7 +2608,7 @@
         <f>AVERAGE(D45:F45)</f>
         <v/>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="H45" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2630,7 +2634,7 @@
           <t>Inverted Spectrum</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -2649,7 +2653,7 @@
         <f>AVERAGE(D46:F46)</f>
         <v/>
       </c>
-      <c r="H46" s="6" t="inlineStr">
+      <c r="H46" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2675,7 +2679,7 @@
           <t>Moral Machine (Self-Driving Car)</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -2698,7 +2702,7 @@
         <f>AVERAGE(D47:F47)</f>
         <v/>
       </c>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="H47" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2724,7 +2728,7 @@
           <t>Newton's Cannonball</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -2743,7 +2747,7 @@
         <f>AVERAGE(D48:F48)</f>
         <v/>
       </c>
-      <c r="H48" s="6" t="inlineStr">
+      <c r="H48" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2769,7 +2773,7 @@
           <t>Russell's Chicken</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -2788,7 +2792,7 @@
         <f>AVERAGE(D49:F49)</f>
         <v/>
       </c>
-      <c r="H49" s="6" t="inlineStr">
+      <c r="H49" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2814,7 +2818,7 @@
           <t>Sorites (Heap)</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -2833,7 +2837,7 @@
         <f>AVERAGE(D50:F50)</f>
         <v/>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="H50" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2859,7 +2863,7 @@
           <t>Stopped Clock</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -2882,7 +2886,7 @@
         <f>AVERAGE(D51:F51)</f>
         <v/>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H51" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2908,7 +2912,7 @@
           <t>Teletransporter</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -2931,7 +2935,7 @@
         <f>AVERAGE(D52:F52)</f>
         <v/>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H52" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -2957,7 +2961,7 @@
           <t>Ticking Time Bomb</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B53" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -2976,7 +2980,7 @@
         <f>AVERAGE(D53:F53)</f>
         <v/>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H53" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3002,7 +3006,7 @@
           <t>Transplant Surgeon</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -3025,7 +3029,7 @@
         <f>AVERAGE(D54:F54)</f>
         <v/>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H54" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3051,7 +3055,7 @@
           <t>Zoo Hypothesis</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -3074,7 +3078,7 @@
         <f>AVERAGE(D55:F55)</f>
         <v/>
       </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="H55" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3100,7 +3104,7 @@
           <t>Cosmological Argument</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -3123,7 +3127,7 @@
         <f>AVERAGE(D56:F56)</f>
         <v/>
       </c>
-      <c r="H56" s="6" t="inlineStr">
+      <c r="H56" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3149,7 +3153,7 @@
           <t>Philosophical Zombie</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -3168,7 +3172,7 @@
         <f>AVERAGE(D57:F57)</f>
         <v/>
       </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="H57" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3194,7 +3198,7 @@
           <t>Veil of Ignorance</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>Political Philosophy</t>
         </is>
@@ -3213,7 +3217,7 @@
         <f>AVERAGE(D58:F58)</f>
         <v/>
       </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="H58" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3239,7 +3243,7 @@
           <t>What Is It Like to Be a Bat?</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -3258,7 +3262,7 @@
         <f>AVERAGE(D59:F59)</f>
         <v/>
       </c>
-      <c r="H59" s="6" t="inlineStr">
+      <c r="H59" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3284,7 +3288,7 @@
           <t>Arrow Paradox</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -3303,7 +3307,7 @@
         <f>AVERAGE(D60:F60)</f>
         <v/>
       </c>
-      <c r="H60" s="6" t="inlineStr">
+      <c r="H60" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3329,7 +3333,7 @@
           <t>Beetle in a Box</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Language</t>
         </is>
@@ -3348,7 +3352,7 @@
         <f>AVERAGE(D61:F61)</f>
         <v/>
       </c>
-      <c r="H61" s="6" t="inlineStr">
+      <c r="H61" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3374,7 +3378,7 @@
           <t>Bootstrap Paradox</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -3393,7 +3397,7 @@
         <f>AVERAGE(D62:F62)</f>
         <v/>
       </c>
-      <c r="H62" s="6" t="inlineStr">
+      <c r="H62" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3419,7 +3423,7 @@
           <t>Einstein's Elevator</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B63" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -3438,7 +3442,7 @@
         <f>AVERAGE(D63:F63)</f>
         <v/>
       </c>
-      <c r="H63" s="6" t="inlineStr">
+      <c r="H63" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3464,7 +3468,7 @@
           <t>Laplace's Demon</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -3483,7 +3487,7 @@
         <f>AVERAGE(D64:F64)</f>
         <v/>
       </c>
-      <c r="H64" s="6" t="inlineStr">
+      <c r="H64" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3509,7 +3513,7 @@
           <t>Library of Babel</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -3528,7 +3532,7 @@
         <f>AVERAGE(D65:F65)</f>
         <v/>
       </c>
-      <c r="H65" s="6" t="inlineStr">
+      <c r="H65" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3554,7 +3558,7 @@
           <t>The Violinist</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -3573,7 +3577,7 @@
         <f>AVERAGE(D66:F66)</f>
         <v/>
       </c>
-      <c r="H66" s="6" t="inlineStr">
+      <c r="H66" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3599,7 +3603,7 @@
           <t>Twin Earth</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Language</t>
         </is>
@@ -3618,7 +3622,7 @@
         <f>AVERAGE(D67:F67)</f>
         <v/>
       </c>
-      <c r="H67" s="6" t="inlineStr">
+      <c r="H67" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3644,7 +3648,7 @@
           <t>Utility Monster</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -3663,7 +3667,7 @@
         <f>AVERAGE(D68:F68)</f>
         <v/>
       </c>
-      <c r="H68" s="6" t="inlineStr">
+      <c r="H68" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3689,7 +3693,7 @@
           <t>Barber Paradox</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -3708,7 +3712,7 @@
         <f>AVERAGE(D69:F69)</f>
         <v/>
       </c>
-      <c r="H69" s="6" t="inlineStr">
+      <c r="H69" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3734,7 +3738,7 @@
           <t>Descartes' Wax</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B70" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -3753,7 +3757,7 @@
         <f>AVERAGE(D70:F70)</f>
         <v/>
       </c>
-      <c r="H70" s="6" t="inlineStr">
+      <c r="H70" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3779,7 +3783,7 @@
           <t>Extended Mind (Otto's Notebook)</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -3798,7 +3802,7 @@
         <f>AVERAGE(D71:F71)</f>
         <v/>
       </c>
-      <c r="H71" s="6" t="inlineStr">
+      <c r="H71" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3824,7 +3828,7 @@
           <t>Gaunilo's Lost Island</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B72" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -3847,7 +3851,7 @@
         <f>AVERAGE(D72:F72)</f>
         <v/>
       </c>
-      <c r="H72" s="6" t="inlineStr">
+      <c r="H72" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3873,7 +3877,7 @@
           <t>Hotelling's Beach</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B73" s="13" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
@@ -3892,7 +3896,7 @@
         <f>AVERAGE(D73:F73)</f>
         <v/>
       </c>
-      <c r="H73" s="6" t="inlineStr">
+      <c r="H73" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3918,7 +3922,7 @@
           <t>Lady Tasting Tea</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -3937,7 +3941,7 @@
         <f>AVERAGE(D74:F74)</f>
         <v/>
       </c>
-      <c r="H74" s="6" t="inlineStr">
+      <c r="H74" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -3963,7 +3967,7 @@
           <t>Lifeboat Ethics</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B75" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -3982,7 +3986,7 @@
         <f>AVERAGE(D75:F75)</f>
         <v/>
       </c>
-      <c r="H75" s="6" t="inlineStr">
+      <c r="H75" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4008,7 +4012,7 @@
           <t>Molyneux's Problem</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B76" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -4027,7 +4031,7 @@
         <f>AVERAGE(D76:F76)</f>
         <v/>
       </c>
-      <c r="H76" s="6" t="inlineStr">
+      <c r="H76" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4053,7 +4057,7 @@
           <t>Neurath's Boat</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B77" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -4072,7 +4076,7 @@
         <f>AVERAGE(D77:F77)</f>
         <v/>
       </c>
-      <c r="H77" s="6" t="inlineStr">
+      <c r="H77" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4098,7 +4102,7 @@
           <t>Prince and the Cobbler</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B78" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -4117,7 +4121,7 @@
         <f>AVERAGE(D78:F78)</f>
         <v/>
       </c>
-      <c r="H78" s="6" t="inlineStr">
+      <c r="H78" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4143,7 +4147,7 @@
           <t>Replaying the Tape of Life</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B79" s="13" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
@@ -4162,7 +4166,7 @@
         <f>AVERAGE(D79:F79)</f>
         <v/>
       </c>
-      <c r="H79" s="6" t="inlineStr">
+      <c r="H79" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4188,7 +4192,7 @@
           <t>Rowe's Fawn</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B80" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -4207,7 +4211,7 @@
         <f>AVERAGE(D80:F80)</f>
         <v/>
       </c>
-      <c r="H80" s="6" t="inlineStr">
+      <c r="H80" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4233,7 +4237,7 @@
           <t>Sheep in the Field</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B81" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -4256,7 +4260,7 @@
         <f>AVERAGE(D81:F81)</f>
         <v/>
       </c>
-      <c r="H81" s="6" t="inlineStr">
+      <c r="H81" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4282,7 +4286,7 @@
           <t>Anthropic Principle / Fine-Tuning</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B82" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -4305,7 +4309,7 @@
         <f>AVERAGE(D82:F82)</f>
         <v/>
       </c>
-      <c r="H82" s="6" t="inlineStr">
+      <c r="H82" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4331,7 +4335,7 @@
           <t>Pascal's Wager</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B83" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -4354,7 +4358,7 @@
         <f>AVERAGE(D83:F83)</f>
         <v/>
       </c>
-      <c r="H83" s="6" t="inlineStr">
+      <c r="H83" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4380,7 +4384,7 @@
           <t>Liar Paradox</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -4399,7 +4403,7 @@
         <f>AVERAGE(D84:F84)</f>
         <v/>
       </c>
-      <c r="H84" s="6" t="inlineStr">
+      <c r="H84" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4425,7 +4429,7 @@
           <t>Boltzmann Brain</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B85" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -4448,7 +4452,7 @@
         <f>AVERAGE(D85:F85)</f>
         <v/>
       </c>
-      <c r="H85" s="6" t="inlineStr">
+      <c r="H85" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4474,7 +4478,7 @@
           <t>Einstein's Train</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B86" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -4493,7 +4497,7 @@
         <f>AVERAGE(D86:F86)</f>
         <v/>
       </c>
-      <c r="H86" s="6" t="inlineStr">
+      <c r="H86" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4519,7 +4523,7 @@
           <t>Kalam Cosmological Argument</t>
         </is>
       </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B87" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -4542,7 +4546,7 @@
         <f>AVERAGE(D87:F87)</f>
         <v/>
       </c>
-      <c r="H87" s="6" t="inlineStr">
+      <c r="H87" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4568,7 +4572,7 @@
           <t>Rare Earth Hypothesis</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B88" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -4591,7 +4595,7 @@
         <f>AVERAGE(D88:F88)</f>
         <v/>
       </c>
-      <c r="H88" s="6" t="inlineStr">
+      <c r="H88" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4617,7 +4621,7 @@
           <t>Roko's Basilisk</t>
         </is>
       </c>
-      <c r="B89" s="3" t="inlineStr">
+      <c r="B89" s="13" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
@@ -4636,7 +4640,7 @@
         <f>AVERAGE(D89:F89)</f>
         <v/>
       </c>
-      <c r="H89" s="6" t="inlineStr">
+      <c r="H89" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4662,7 +4666,7 @@
           <t>Barn Façade County</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -4685,7 +4689,7 @@
         <f>AVERAGE(D90:F90)</f>
         <v/>
       </c>
-      <c r="H90" s="6" t="inlineStr">
+      <c r="H90" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4711,7 +4715,7 @@
           <t>China Brain</t>
         </is>
       </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="B91" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -4730,7 +4734,7 @@
         <f>AVERAGE(D91:F91)</f>
         <v/>
       </c>
-      <c r="H91" s="6" t="inlineStr">
+      <c r="H91" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4756,7 +4760,7 @@
           <t>Floating Man</t>
         </is>
       </c>
-      <c r="B92" s="3" t="inlineStr">
+      <c r="B92" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -4775,7 +4779,7 @@
         <f>AVERAGE(D92:F92)</f>
         <v/>
       </c>
-      <c r="H92" s="6" t="inlineStr">
+      <c r="H92" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4801,7 +4805,7 @@
           <t>Galileo's Ship</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B93" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -4820,7 +4824,7 @@
         <f>AVERAGE(D93:F93)</f>
         <v/>
       </c>
-      <c r="H93" s="6" t="inlineStr">
+      <c r="H93" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4846,7 +4850,7 @@
           <t>Keynesian Beauty Contest</t>
         </is>
       </c>
-      <c r="B94" s="3" t="inlineStr">
+      <c r="B94" s="13" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
@@ -4865,7 +4869,7 @@
         <f>AVERAGE(D94:F94)</f>
         <v/>
       </c>
-      <c r="H94" s="6" t="inlineStr">
+      <c r="H94" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4891,7 +4895,7 @@
           <t>Leibniz's Mill</t>
         </is>
       </c>
-      <c r="B95" s="3" t="inlineStr">
+      <c r="B95" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -4910,7 +4914,7 @@
         <f>AVERAGE(D95:F95)</f>
         <v/>
       </c>
-      <c r="H95" s="6" t="inlineStr">
+      <c r="H95" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4936,7 +4940,7 @@
           <t>Meno's Slave Boy</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B96" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -4955,7 +4959,7 @@
         <f>AVERAGE(D96:F96)</f>
         <v/>
       </c>
-      <c r="H96" s="6" t="inlineStr">
+      <c r="H96" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -4981,7 +4985,7 @@
           <t>Missing Shade of Blue</t>
         </is>
       </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="B97" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -5000,7 +5004,7 @@
         <f>AVERAGE(D97:F97)</f>
         <v/>
       </c>
-      <c r="H97" s="6" t="inlineStr">
+      <c r="H97" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5026,7 +5030,7 @@
           <t>Olbers' Paradox</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B98" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -5045,7 +5049,7 @@
         <f>AVERAGE(D98:F98)</f>
         <v/>
       </c>
-      <c r="H98" s="6" t="inlineStr">
+      <c r="H98" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5071,7 +5075,7 @@
           <t>Quantum Suicide</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B99" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -5090,7 +5094,7 @@
         <f>AVERAGE(D99:F99)</f>
         <v/>
       </c>
-      <c r="H99" s="6" t="inlineStr">
+      <c r="H99" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5116,7 +5120,7 @@
           <t>Swampman</t>
         </is>
       </c>
-      <c r="B100" s="3" t="inlineStr">
+      <c r="B100" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Mind</t>
         </is>
@@ -5139,7 +5143,7 @@
         <f>AVERAGE(D100:F100)</f>
         <v/>
       </c>
-      <c r="H100" s="6" t="inlineStr">
+      <c r="H100" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5165,7 +5169,7 @@
           <t>Dawkins' Weasel</t>
         </is>
       </c>
-      <c r="B101" s="3" t="inlineStr">
+      <c r="B101" s="13" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
@@ -5184,7 +5188,7 @@
         <f>AVERAGE(D101:F101)</f>
         <v/>
       </c>
-      <c r="H101" s="6" t="inlineStr">
+      <c r="H101" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5210,7 +5214,7 @@
           <t>Stag Hunt</t>
         </is>
       </c>
-      <c r="B102" s="3" t="inlineStr">
+      <c r="B102" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -5229,7 +5233,7 @@
         <f>AVERAGE(D102:F102)</f>
         <v/>
       </c>
-      <c r="H102" s="6" t="inlineStr">
+      <c r="H102" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5255,7 +5259,7 @@
           <t>Dharmottara's Mirage</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B103" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -5278,7 +5282,7 @@
         <f>AVERAGE(D103:F103)</f>
         <v/>
       </c>
-      <c r="H103" s="6" t="inlineStr">
+      <c r="H103" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5304,7 +5308,7 @@
           <t>Ontological Argument</t>
         </is>
       </c>
-      <c r="B104" s="3" t="inlineStr">
+      <c r="B104" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Religion &amp; Ontology</t>
         </is>
@@ -5327,7 +5331,7 @@
         <f>AVERAGE(D104:F104)</f>
         <v/>
       </c>
-      <c r="H104" s="6" t="inlineStr">
+      <c r="H104" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5353,7 +5357,7 @@
           <t>Banach–Tarski Paradox</t>
         </is>
       </c>
-      <c r="B105" s="3" t="inlineStr">
+      <c r="B105" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -5372,7 +5376,7 @@
         <f>AVERAGE(D105:F105)</f>
         <v/>
       </c>
-      <c r="H105" s="6" t="inlineStr">
+      <c r="H105" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5398,7 +5402,7 @@
           <t>Newcomb's Paradox</t>
         </is>
       </c>
-      <c r="B106" s="3" t="inlineStr">
+      <c r="B106" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -5417,7 +5421,7 @@
         <f>AVERAGE(D106:F106)</f>
         <v/>
       </c>
-      <c r="H106" s="6" t="inlineStr">
+      <c r="H106" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5443,7 +5447,7 @@
           <t>Gettier Problem</t>
         </is>
       </c>
-      <c r="B107" s="3" t="inlineStr">
+      <c r="B107" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -5466,7 +5470,7 @@
         <f>AVERAGE(D107:F107)</f>
         <v/>
       </c>
-      <c r="H107" s="6" t="inlineStr">
+      <c r="H107" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5492,7 +5496,7 @@
           <t>Gabriel's Horn</t>
         </is>
       </c>
-      <c r="B108" s="3" t="inlineStr">
+      <c r="B108" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -5511,7 +5515,7 @@
         <f>AVERAGE(D108:F108)</f>
         <v/>
       </c>
-      <c r="H108" s="6" t="inlineStr">
+      <c r="H108" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5537,7 +5541,7 @@
           <t>Heisenberg's Microscope</t>
         </is>
       </c>
-      <c r="B109" s="3" t="inlineStr">
+      <c r="B109" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -5556,7 +5560,7 @@
         <f>AVERAGE(D109:F109)</f>
         <v/>
       </c>
-      <c r="H109" s="6" t="inlineStr">
+      <c r="H109" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5582,7 +5586,7 @@
           <t>Ladder Paradox</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B110" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -5601,7 +5605,7 @@
         <f>AVERAGE(D110:F110)</f>
         <v/>
       </c>
-      <c r="H110" s="6" t="inlineStr">
+      <c r="H110" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5627,7 +5631,7 @@
           <t>Loop Track</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B111" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -5650,7 +5654,7 @@
         <f>AVERAGE(D111:F111)</f>
         <v/>
       </c>
-      <c r="H111" s="6" t="inlineStr">
+      <c r="H111" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5676,7 +5680,7 @@
           <t>Newton's Bucket</t>
         </is>
       </c>
-      <c r="B112" s="3" t="inlineStr">
+      <c r="B112" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -5695,7 +5699,7 @@
         <f>AVERAGE(D112:F112)</f>
         <v/>
       </c>
-      <c r="H112" s="6" t="inlineStr">
+      <c r="H112" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5721,7 +5725,7 @@
           <t>Wigner's Friend</t>
         </is>
       </c>
-      <c r="B113" s="3" t="inlineStr">
+      <c r="B113" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -5740,7 +5744,7 @@
         <f>AVERAGE(D113:F113)</f>
         <v/>
       </c>
-      <c r="H113" s="6" t="inlineStr">
+      <c r="H113" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5766,7 +5770,7 @@
           <t>Gavagai</t>
         </is>
       </c>
-      <c r="B114" s="3" t="inlineStr">
+      <c r="B114" s="13" t="inlineStr">
         <is>
           <t>Philosophy of Language</t>
         </is>
@@ -5785,7 +5789,7 @@
         <f>AVERAGE(D114:F114)</f>
         <v/>
       </c>
-      <c r="H114" s="6" t="inlineStr">
+      <c r="H114" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5811,7 +5815,7 @@
           <t>Moral Luck (Two Drivers)</t>
         </is>
       </c>
-      <c r="B115" s="3" t="inlineStr">
+      <c r="B115" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -5830,7 +5834,7 @@
         <f>AVERAGE(D115:F115)</f>
         <v/>
       </c>
-      <c r="H115" s="6" t="inlineStr">
+      <c r="H115" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5856,7 +5860,7 @@
           <t>Pascal's Mugging</t>
         </is>
       </c>
-      <c r="B116" s="3" t="inlineStr">
+      <c r="B116" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -5879,7 +5883,7 @@
         <f>AVERAGE(D116:F116)</f>
         <v/>
       </c>
-      <c r="H116" s="6" t="inlineStr">
+      <c r="H116" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5905,7 +5909,7 @@
           <t>Unexpected Hanging</t>
         </is>
       </c>
-      <c r="B117" s="3" t="inlineStr">
+      <c r="B117" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -5924,7 +5928,7 @@
         <f>AVERAGE(D117:F117)</f>
         <v/>
       </c>
-      <c r="H117" s="6" t="inlineStr">
+      <c r="H117" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5950,7 +5954,7 @@
           <t>Wilt Chamberlain Argument</t>
         </is>
       </c>
-      <c r="B118" s="3" t="inlineStr">
+      <c r="B118" s="13" t="inlineStr">
         <is>
           <t>Political Philosophy</t>
         </is>
@@ -5969,7 +5973,7 @@
         <f>AVERAGE(D118:F118)</f>
         <v/>
       </c>
-      <c r="H118" s="6" t="inlineStr">
+      <c r="H118" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -5995,7 +5999,7 @@
           <t>Stevin's Chain</t>
         </is>
       </c>
-      <c r="B119" s="3" t="inlineStr">
+      <c r="B119" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -6014,7 +6018,7 @@
         <f>AVERAGE(D119:F119)</f>
         <v/>
       </c>
-      <c r="H119" s="6" t="inlineStr">
+      <c r="H119" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6040,7 +6044,7 @@
           <t>Thomson's Lamp</t>
         </is>
       </c>
-      <c r="B120" s="3" t="inlineStr">
+      <c r="B120" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -6059,7 +6063,7 @@
         <f>AVERAGE(D120:F120)</f>
         <v/>
       </c>
-      <c r="H120" s="6" t="inlineStr">
+      <c r="H120" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6085,7 +6089,7 @@
           <t>Doomsday Argument</t>
         </is>
       </c>
-      <c r="B121" s="3" t="inlineStr">
+      <c r="B121" s="13" t="inlineStr">
         <is>
           <t>Cosmology &amp; Astrobiology</t>
         </is>
@@ -6104,7 +6108,7 @@
         <f>AVERAGE(D121:F121)</f>
         <v/>
       </c>
-      <c r="H121" s="6" t="inlineStr">
+      <c r="H121" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6130,7 +6134,7 @@
           <t>Grue</t>
         </is>
       </c>
-      <c r="B122" s="3" t="inlineStr">
+      <c r="B122" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -6149,7 +6153,7 @@
         <f>AVERAGE(D122:F122)</f>
         <v/>
       </c>
-      <c r="H122" s="6" t="inlineStr">
+      <c r="H122" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6175,7 +6179,7 @@
           <t>Raven Paradox</t>
         </is>
       </c>
-      <c r="B123" s="3" t="inlineStr">
+      <c r="B123" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -6194,7 +6198,7 @@
         <f>AVERAGE(D123:F123)</f>
         <v/>
       </c>
-      <c r="H123" s="6" t="inlineStr">
+      <c r="H123" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6220,7 +6224,7 @@
           <t>Repugnant Conclusion</t>
         </is>
       </c>
-      <c r="B124" s="3" t="inlineStr">
+      <c r="B124" s="13" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
@@ -6239,7 +6243,7 @@
         <f>AVERAGE(D124:F124)</f>
         <v/>
       </c>
-      <c r="H124" s="6" t="inlineStr">
+      <c r="H124" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6265,7 +6269,7 @@
           <t>Sleeping Beauty Problem</t>
         </is>
       </c>
-      <c r="B125" s="3" t="inlineStr">
+      <c r="B125" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -6284,7 +6288,7 @@
         <f>AVERAGE(D125:F125)</f>
         <v/>
       </c>
-      <c r="H125" s="6" t="inlineStr">
+      <c r="H125" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6310,7 +6314,7 @@
           <t>Ten Coins in the Pocket</t>
         </is>
       </c>
-      <c r="B126" s="3" t="inlineStr">
+      <c r="B126" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -6333,7 +6337,7 @@
         <f>AVERAGE(D126:F126)</f>
         <v/>
       </c>
-      <c r="H126" s="6" t="inlineStr">
+      <c r="H126" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6359,7 +6363,7 @@
           <t>Two Envelopes Problem</t>
         </is>
       </c>
-      <c r="B127" s="3" t="inlineStr">
+      <c r="B127" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -6378,7 +6382,7 @@
         <f>AVERAGE(D127:F127)</f>
         <v/>
       </c>
-      <c r="H127" s="6" t="inlineStr">
+      <c r="H127" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6404,7 +6408,7 @@
           <t>Black's Two Spheres</t>
         </is>
       </c>
-      <c r="B128" s="3" t="inlineStr">
+      <c r="B128" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -6423,7 +6427,7 @@
         <f>AVERAGE(D128:F128)</f>
         <v/>
       </c>
-      <c r="H128" s="6" t="inlineStr">
+      <c r="H128" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6449,7 +6453,7 @@
           <t>Brownian Ratchet</t>
         </is>
       </c>
-      <c r="B129" s="3" t="inlineStr">
+      <c r="B129" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -6468,7 +6472,7 @@
         <f>AVERAGE(D129:F129)</f>
         <v/>
       </c>
-      <c r="H129" s="6" t="inlineStr">
+      <c r="H129" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6494,7 +6498,7 @@
           <t>Ross–Littlewood Paradox</t>
         </is>
       </c>
-      <c r="B130" s="3" t="inlineStr">
+      <c r="B130" s="13" t="inlineStr">
         <is>
           <t>Logic &amp; Mathematics</t>
         </is>
@@ -6513,7 +6517,7 @@
         <f>AVERAGE(D130:F130)</f>
         <v/>
       </c>
-      <c r="H130" s="6" t="inlineStr">
+      <c r="H130" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6539,7 +6543,7 @@
           <t>EPR Paradox</t>
         </is>
       </c>
-      <c r="B131" s="3" t="inlineStr">
+      <c r="B131" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -6558,7 +6562,7 @@
         <f>AVERAGE(D131:F131)</f>
         <v/>
       </c>
-      <c r="H131" s="6" t="inlineStr">
+      <c r="H131" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6584,7 +6588,7 @@
           <t>Frankfurt Cases</t>
         </is>
       </c>
-      <c r="B132" s="3" t="inlineStr">
+      <c r="B132" s="13" t="inlineStr">
         <is>
           <t>Metaphysics</t>
         </is>
@@ -6603,7 +6607,7 @@
         <f>AVERAGE(D132:F132)</f>
         <v/>
       </c>
-      <c r="H132" s="6" t="inlineStr">
+      <c r="H132" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6629,7 +6633,7 @@
           <t>St. Petersburg Paradox</t>
         </is>
       </c>
-      <c r="B133" s="3" t="inlineStr">
+      <c r="B133" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -6648,7 +6652,7 @@
         <f>AVERAGE(D133:F133)</f>
         <v/>
       </c>
-      <c r="H133" s="6" t="inlineStr">
+      <c r="H133" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6674,7 +6678,7 @@
           <t>Bell's Spaceship Paradox</t>
         </is>
       </c>
-      <c r="B134" s="3" t="inlineStr">
+      <c r="B134" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -6693,7 +6697,7 @@
         <f>AVERAGE(D134:F134)</f>
         <v/>
       </c>
-      <c r="H134" s="6" t="inlineStr">
+      <c r="H134" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6719,7 +6723,7 @@
           <t>Kavka's Toxin Puzzle</t>
         </is>
       </c>
-      <c r="B135" s="3" t="inlineStr">
+      <c r="B135" s="13" t="inlineStr">
         <is>
           <t>Decision Theory, Game Theory &amp; Probability</t>
         </is>
@@ -6738,7 +6742,7 @@
         <f>AVERAGE(D135:F135)</f>
         <v/>
       </c>
-      <c r="H135" s="6" t="inlineStr">
+      <c r="H135" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6764,7 +6768,7 @@
           <t>Lottery Paradox</t>
         </is>
       </c>
-      <c r="B136" s="3" t="inlineStr">
+      <c r="B136" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -6783,7 +6787,7 @@
         <f>AVERAGE(D136:F136)</f>
         <v/>
       </c>
-      <c r="H136" s="6" t="inlineStr">
+      <c r="H136" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6809,7 +6813,7 @@
           <t>Ford or Barcelona</t>
         </is>
       </c>
-      <c r="B137" s="3" t="inlineStr">
+      <c r="B137" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -6832,7 +6836,7 @@
         <f>AVERAGE(D137:F137)</f>
         <v/>
       </c>
-      <c r="H137" s="6" t="inlineStr">
+      <c r="H137" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6858,7 +6862,7 @@
           <t>Nogot and Havit</t>
         </is>
       </c>
-      <c r="B138" s="3" t="inlineStr">
+      <c r="B138" s="13" t="inlineStr">
         <is>
           <t>Epistemology</t>
         </is>
@@ -6881,7 +6885,7 @@
         <f>AVERAGE(D138:F138)</f>
         <v/>
       </c>
-      <c r="H138" s="6" t="inlineStr">
+      <c r="H138" s="14" t="inlineStr">
         <is>
           <t>Wikipedia</t>
         </is>
@@ -6916,222 +6920,223 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I117" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I122" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I124" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I126" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I131" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I132" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I138" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I117" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I122" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I124" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I126" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I131" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I132" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I138" r:id="rId219"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Make the repo the game; archive the films
- The engine the game runs on moves to game/engine/ (core.js trimmed of the
  film-only timeline, camera paths, captions and overlays; style.css cut
  down to what the game uses). All imports updated.
- The films go to archive/films/: experiments/, the renderer (render.mjs,
  player.html), PRODUCTION.md, sfx.py, with a README. Tag films-v1 keeps the
  working film pipeline.
- What the game needed from the films is folded in: Brain in a Vat's lab
  models (game/core/lab.js), the two notebooks (game/notebook/), and
  PRODUCTION.md's standards (GAME.md §8: research, writing, visual
  language, voice and the narration audit, pitfalls).
- tools/audit.py now audits a vignette's voice lines; setup.sh and
  package.json are about playing and voicing the game.
- README is about the game; the spreadsheet's 'Video created' column is
  now 'In the game' (18 ticked).
- game/tools/smoke.mjs loads every room and vignette and reports errors.
</commit_message>
<xml_diff>
--- a/thought_experiments.xlsx
+++ b/thought_experiments.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Video created</t>
+          <t>In the game</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="K3" s="13" t="n"/>
       <c r="L3" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -732,7 +732,7 @@
       </c>
       <c r="K4" s="13" t="n"/>
       <c r="L4" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -777,7 +777,7 @@
       </c>
       <c r="K5" s="13" t="n"/>
       <c r="L5" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -822,7 +822,7 @@
       </c>
       <c r="K6" s="13" t="n"/>
       <c r="L6" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -871,7 +871,7 @@
       </c>
       <c r="K7" s="13" t="n"/>
       <c r="L7" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -920,7 +920,7 @@
       </c>
       <c r="K8" s="13" t="n"/>
       <c r="L8" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -965,7 +965,7 @@
       </c>
       <c r="K9" s="13" t="n"/>
       <c r="L9" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="K12" s="13" t="n"/>
       <c r="L12" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="K13" s="13" t="n"/>
       <c r="L13" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="K15" s="13" t="n"/>
       <c r="L15" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="K22" s="13" t="n"/>
       <c r="L22" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="K27" s="13" t="n"/>
       <c r="L27" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="K54" s="13" t="n"/>
       <c r="L54" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="K68" s="13" t="n"/>
       <c r="L68" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -5438,7 +5438,7 @@
       </c>
       <c r="K106" s="13" t="n"/>
       <c r="L106" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="K111" s="13" t="n"/>
       <c r="L111" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -7418,7 +7418,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Mean of the three ratings. The main sheet is sorted by it, highest first, so we make the films in that order.</t>
+          <t>Mean of the three ratings. The main sheet is sorted by it, highest first, so we build the vignettes in that order.</t>
         </is>
       </c>
     </row>
@@ -7538,19 +7538,19 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Link to an in-depth video essay by another creator, recommended in the video description.</t>
+          <t>Link to an in-depth video essay by another creator. It goes in the vignette's notebook and the journal's to-do list.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Video created</t>
+          <t>In the game</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>TRUE once the film is rendered and in experiments/&lt;id&gt;/ in the repo. Rows turn green when TRUE.</t>
+          <t>TRUE once the vignette is playable in the game (game/vignettes/&lt;id&gt;.js). Rows turn green when TRUE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The field and the barn in GAME.md and the README; the spreadsheet marks all fifteen as in the game; the field's camera sits a little higher; Omelas said as Le Guin said it; the fastest lines slowed; playtests for the field and the barn
</commit_message>
<xml_diff>
--- a/thought_experiments.xlsx
+++ b/thought_experiments.xlsx
@@ -1517,7 +1517,7 @@
       </c>
       <c r="K21" s="13" t="n"/>
       <c r="L21" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="K24" s="13" t="n"/>
       <c r="L24" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="K25" s="13" t="n"/>
       <c r="L25" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="K26" s="13" t="n"/>
       <c r="L26" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="K29" s="13" t="n"/>
       <c r="L29" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="K30" s="13" t="n"/>
       <c r="L30" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="K42" s="13" t="n"/>
       <c r="L42" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="K51" s="13" t="n"/>
       <c r="L51" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="K58" s="13" t="n"/>
       <c r="L58" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="K81" s="13" t="n"/>
       <c r="L81" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="K90" s="13" t="n"/>
       <c r="L90" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="K100" s="13" t="n"/>
       <c r="L100" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -5299,7 +5299,7 @@
       </c>
       <c r="K103" s="13" t="n"/>
       <c r="L103" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="K107" s="13" t="n"/>
       <c r="L107" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -6354,7 +6354,7 @@
       </c>
       <c r="K126" s="13" t="n"/>
       <c r="L126" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127">

</xml_diff>